<commit_message>
state of health report (mostly)
</commit_message>
<xml_diff>
--- a/myAnalyses/0.StateOfHealth/raceAgeExplore1.xlsx
+++ b/myAnalyses/0.StateOfHealth/raceAgeExplore1.xlsx
@@ -211,9 +211,6 @@
     <t>Substance use disorders</t>
   </si>
   <si>
-    <t>Alzheimerâ€™s disease and other dementias</t>
-  </si>
-  <si>
     <t>Other neurological conditions</t>
   </si>
   <si>
@@ -290,6 +287,9 @@
   </si>
   <si>
     <t>Crude Rates and Numbers of Deaths by Cause, by Race/Ethnic Group, with black to white percent comparison</t>
+  </si>
+  <si>
+    <t>Alzheimer's disease and other dementias</t>
   </si>
 </sst>
 </file>
@@ -1154,17 +1154,17 @@
   <sheetData>
     <row r="1" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
@@ -1172,7 +1172,7 @@
         <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C5" s="2">
         <v>494.79104664171501</v>
@@ -1281,7 +1281,7 @@
         <v>7</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>8</v>
@@ -1302,7 +1302,7 @@
         <v>13</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="Q7" t="s">
         <v>14</v>
@@ -1346,7 +1346,7 @@
         <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="C8" s="2">
         <v>3.8513026981534502</v>
@@ -1389,7 +1389,7 @@
         <v>1179.5275795257901</v>
       </c>
       <c r="P8" s="3">
-        <f t="shared" ref="P8:P65" si="1">(L8-O8)/O8</f>
+        <f t="shared" ref="P8:P62" si="1">(L8-O8)/O8</f>
         <v>-0.1212785885777351</v>
       </c>
       <c r="Q8">
@@ -1610,7 +1610,7 @@
         <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C11" s="2">
         <v>21.0808147688399</v>
@@ -2050,7 +2050,7 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C16" s="2">
         <v>7.0945049702826797</v>
@@ -2314,7 +2314,7 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C19" s="2">
         <v>7.0945049702826797</v>
@@ -2402,7 +2402,7 @@
         <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C20" s="2">
         <v>19.256513490767201</v>
@@ -2490,7 +2490,7 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C21" s="2">
         <v>7.7026053963069101</v>
@@ -2578,7 +2578,7 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C22" s="2">
         <v>8.1080056803230693</v>
@@ -3194,7 +3194,7 @@
         <v>26</v>
       </c>
       <c r="B29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C29" s="2">
         <v>1.6216011360646101</v>
@@ -3722,7 +3722,7 @@
         <v>26</v>
       </c>
       <c r="B35" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C35" s="2">
         <v>42.567029821696103</v>
@@ -3986,7 +3986,7 @@
         <v>26</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C38" s="2">
         <v>7.4999052542988398</v>
@@ -4338,7 +4338,7 @@
         <v>26</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C42" s="2">
         <v>15.202510650605699</v>
@@ -4778,7 +4778,7 @@
         <v>26</v>
       </c>
       <c r="B47" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C47" s="2">
         <v>20.270014200807601</v>
@@ -4866,7 +4866,7 @@
         <v>26</v>
       </c>
       <c r="B48" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C48" s="2">
         <v>6.0810042602422998</v>
@@ -4954,7 +4954,7 @@
         <v>26</v>
       </c>
       <c r="B49" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C49" s="2">
         <v>1.0135007100403799</v>
@@ -5218,7 +5218,7 @@
         <v>26</v>
       </c>
       <c r="B52" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C52" s="2">
         <v>1.41890099405653</v>
@@ -5394,7 +5394,7 @@
         <v>26</v>
       </c>
       <c r="B54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C54" s="2">
         <v>0.40540028401615302</v>
@@ -5482,7 +5482,7 @@
         <v>26</v>
       </c>
       <c r="B55" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C55" s="2">
         <v>29.796920875187201</v>
@@ -5570,7 +5570,7 @@
         <v>26</v>
       </c>
       <c r="B56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C56" s="2">
         <v>10.5404073844199</v>
@@ -5834,7 +5834,7 @@
         <v>26</v>
       </c>
       <c r="B59" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C59" s="2">
         <v>4.1666915455611102</v>
@@ -5859,7 +5859,7 @@
         <v>-0.11847384256693104</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K59" s="2">
         <v>0.66998548543792902</v>
@@ -5871,7 +5871,7 @@
         <v>0.68714995886279795</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O59" s="2">
         <v>0.67677811940004895</v>
@@ -5899,7 +5899,7 @@
         <v>353</v>
       </c>
       <c r="W59" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="X59">
         <v>7</v>
@@ -5911,7 +5911,7 @@
         <v>9</v>
       </c>
       <c r="AA59" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AB59">
         <v>28</v>
@@ -6098,7 +6098,7 @@
         <v>26</v>
       </c>
       <c r="B62" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C62" s="2">
         <v>0.20270014200807601</v>
@@ -6229,7 +6229,7 @@
         <v>0</v>
       </c>
       <c r="P63" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Q63">
         <v>10</v>
@@ -6316,7 +6316,7 @@
         <v>0</v>
       </c>
       <c r="P64" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Q64">
         <v>0</v>
@@ -6360,29 +6360,29 @@
         <v>26</v>
       </c>
       <c r="B65" t="s">
+        <v>83</v>
+      </c>
+      <c r="C65" s="2">
+        <v>0</v>
+      </c>
+      <c r="D65" s="2">
+        <v>0</v>
+      </c>
+      <c r="E65" s="2">
+        <v>0</v>
+      </c>
+      <c r="F65" s="2">
+        <v>0</v>
+      </c>
+      <c r="G65" s="2">
+        <v>0</v>
+      </c>
+      <c r="H65" s="2">
+        <v>0</v>
+      </c>
+      <c r="I65" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C65" s="2">
-        <v>0</v>
-      </c>
-      <c r="D65" s="2">
-        <v>0</v>
-      </c>
-      <c r="E65" s="2">
-        <v>0</v>
-      </c>
-      <c r="F65" s="2">
-        <v>0</v>
-      </c>
-      <c r="G65" s="2">
-        <v>0</v>
-      </c>
-      <c r="H65" s="2">
-        <v>0</v>
-      </c>
-      <c r="I65" s="3" t="s">
-        <v>85</v>
-      </c>
       <c r="J65" s="2">
         <v>0</v>
       </c>
@@ -6402,7 +6402,7 @@
         <v>0</v>
       </c>
       <c r="P65" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Q65">
         <v>0</v>

</xml_diff>